<commit_message>
Deployed 676377ac to update-tests with MkDocs 1.6.1 and mike 2.2.0
</commit_message>
<xml_diff>
--- a/update-tests/catalog_summary.xlsx
+++ b/update-tests/catalog_summary.xlsx
@@ -8981,12 +8981,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
+          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
+          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -8996,7 +8996,7 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
+          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F77" t="inlineStr">
@@ -9012,7 +9012,11 @@
       <c r="H77" t="b">
         <v>0</v>
       </c>
-      <c r="I77" t="inlineStr"/>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>Airborne Coastal Observatory</t>
+        </is>
+      </c>
       <c r="J77" t="inlineStr">
         <is>
           <t>completed</t>
@@ -9038,12 +9042,12 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
         </is>
       </c>
       <c r="P77" t="inlineStr">
         <is>
-          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q77" t="inlineStr">
@@ -9054,7 +9058,7 @@
       <c r="R77" t="inlineStr"/>
       <c r="S77" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
         </is>
       </c>
       <c r="T77" t="inlineStr">
@@ -9068,7 +9072,7 @@
         </is>
       </c>
       <c r="V77" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="W77" t="inlineStr"/>
       <c r="X77" t="inlineStr"/>
@@ -9080,12 +9084,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>92e1c9df-0419-4d91-93c2-b9c85f4ce74e</t>
+          <t>8a71bb9f-e419-42aa-9ed7-f891631314a5</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>ca-cioos_0f524f76-a88b-4e0a-9c3c-ee83114c3679</t>
+          <t>ca-cioos_0ebfdd89-61d6-453c-870a-83167617b26a</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -9095,7 +9099,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Gitanyow Archaeology, Cranberry Junction - 2020 - Airborne Coastal Observatory</t>
+          <t>Glacier and Icefield Mapping - British Columbia - 2019 - Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="F78" t="inlineStr">
@@ -9111,11 +9115,7 @@
       <c r="H78" t="b">
         <v>0</v>
       </c>
-      <c r="I78" t="inlineStr">
-        <is>
-          <t>Airborne Coastal Observatory</t>
-        </is>
-      </c>
+      <c r="I78" t="inlineStr"/>
       <c r="J78" t="inlineStr">
         <is>
           <t>completed</t>
@@ -9141,12 +9141,12 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.0, 55.96], [-127.2, 55.96], [-127.2, 56.36], [-128.0, 56.36], [-128.0, 55.96]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-127.4, 48.85], [-114.4, 48.85], [-114.4, 55.75], [-127.4, 55.75], [-127.4, 48.85]]]}</t>
         </is>
       </c>
       <c r="P78" t="inlineStr">
         <is>
-          <t>[{'max': '1000.0', 'min': '0.0'}]</t>
+          <t>[{'max': '2000.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q78" t="inlineStr">
@@ -9157,7 +9157,7 @@
       <c r="R78" t="inlineStr"/>
       <c r="S78" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MiNpB5mjvTnWKqOFiq-</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/RvRPlFMSsIaBwoGdQIq5BVYfBBa2/-MkE_rRkw9irKz8XxrLV</t>
         </is>
       </c>
       <c r="T78" t="inlineStr">
@@ -9171,7 +9171,7 @@
         </is>
       </c>
       <c r="V78" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="W78" t="inlineStr"/>
       <c r="X78" t="inlineStr"/>
@@ -15783,12 +15783,12 @@
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
+          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
+          <t>ca-cioos_a242acd4-e3c7-46e0-8f43-f428fb824018</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
@@ -15798,7 +15798,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
+          <t>Stage-Discharge Time Series - Calvert Island - Archived Version 1.0</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
@@ -15816,7 +15816,7 @@
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>Airborne Coastal Observatory</t>
+          <t>Watersheds</t>
         </is>
       </c>
       <c r="J139" t="inlineStr">
@@ -15836,20 +15836,20 @@
       </c>
       <c r="M139" t="inlineStr">
         <is>
-          <t>University of Victoria</t>
+          <t>Vancouver Island University</t>
         </is>
       </c>
       <c r="N139" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O139" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.13217163085935, 51.59626804559349], [-127.97149658203124, 51.59626804559349], [-127.97149658203124, 51.6857538480987], [-128.13217163085935, 51.6857538480987], [-128.13217163085935, 51.59626804559349]]]}</t>
         </is>
       </c>
       <c r="P139" t="inlineStr">
         <is>
-          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
+          <t>[{'max': '250.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q139" t="inlineStr">
@@ -15857,14 +15857,10 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R139" t="inlineStr">
-        <is>
-          <t>10.21966/1.135248</t>
-        </is>
-      </c>
+      <c r="R139" t="inlineStr"/>
       <c r="S139" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpNR0VhOVRlU210cDI</t>
         </is>
       </c>
       <c r="T139" t="inlineStr">
@@ -15874,25 +15870,15 @@
       </c>
       <c r="U139" t="inlineStr">
         <is>
-          <t>2024-07-24</t>
+          <t>2024-12-05</t>
         </is>
       </c>
       <c r="V139" t="n">
-        <v>2</v>
-      </c>
-      <c r="W139" t="n">
-        <v>0</v>
-      </c>
-      <c r="X139" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
-      <c r="Y139" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="W139" t="inlineStr"/>
+      <c r="X139" t="inlineStr"/>
+      <c r="Y139" t="inlineStr"/>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -15900,12 +15886,12 @@
       </c>
       <c r="B140" t="inlineStr">
         <is>
-          <t>6f261f49-dd1b-4250-ac59-e88c3d1b2470</t>
+          <t>18911dee-9ca0-408b-8999-28da3e3dde7a</t>
         </is>
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>ca-cioos_a242acd4-e3c7-46e0-8f43-f428fb824018</t>
+          <t>ca-cioos_9e61819e-8385-41d2-a5c5-0e2f37c522ef</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
@@ -15915,7 +15901,7 @@
       </c>
       <c r="E140" t="inlineStr">
         <is>
-          <t>Stage-Discharge Time Series - Calvert Island - Archived Version 1.0</t>
+          <t>LiDAR-based Ecosystem Classification for Calvert Island</t>
         </is>
       </c>
       <c r="F140" t="inlineStr">
@@ -15933,7 +15919,7 @@
       </c>
       <c r="I140" t="inlineStr">
         <is>
-          <t>Watersheds</t>
+          <t>Airborne Coastal Observatory</t>
         </is>
       </c>
       <c r="J140" t="inlineStr">
@@ -15953,20 +15939,20 @@
       </c>
       <c r="M140" t="inlineStr">
         <is>
-          <t>Vancouver Island University</t>
+          <t>University of Victoria</t>
         </is>
       </c>
       <c r="N140" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O140" t="inlineStr">
         <is>
-          <t>{'type': 'Polygon', 'coordinates': [[[-128.13217163085935, 51.59626804559349], [-127.97149658203124, 51.59626804559349], [-127.97149658203124, 51.6857538480987], [-128.13217163085935, 51.6857538480987], [-128.13217163085935, 51.59626804559349]]]}</t>
+          <t>{'type': 'Polygon', 'coordinates': [[[-128.22692871093747, 51.40948589555509], [-127.80944824218746, 51.40948589555509], [-127.80944824218746, 51.74233687689102], [-128.22692871093747, 51.74233687689102], [-128.22692871093747, 51.40948589555509]]]}</t>
         </is>
       </c>
       <c r="P140" t="inlineStr">
         <is>
-          <t>[{'max': '250.0', 'min': '0.0'}]</t>
+          <t>[{'max': '1014.0', 'min': '0.0'}]</t>
         </is>
       </c>
       <c r="Q140" t="inlineStr">
@@ -15974,10 +15960,14 @@
           <t>other</t>
         </is>
       </c>
-      <c r="R140" t="inlineStr"/>
+      <c r="R140" t="inlineStr">
+        <is>
+          <t>10.21966/1.135248</t>
+        </is>
+      </c>
       <c r="S140" t="inlineStr">
         <is>
-          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MUpNR0VhOVRlU210cDI</t>
+          <t>https://hakaiinstitute.github.io/hakai-metadata-entry-form#/en/hakai/qbqh6DF00XZq8MOpQ3kKkI9GUv43/-MVFjSmdJMGxrU1pZbXM</t>
         </is>
       </c>
       <c r="T140" t="inlineStr">
@@ -15987,15 +15977,25 @@
       </c>
       <c r="U140" t="inlineStr">
         <is>
-          <t>2024-12-05</t>
+          <t>2024-07-24</t>
         </is>
       </c>
       <c r="V140" t="n">
-        <v>5</v>
-      </c>
-      <c r="W140" t="inlineStr"/>
-      <c r="X140" t="inlineStr"/>
-      <c r="Y140" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="W140" t="n">
+        <v>0</v>
+      </c>
+      <c r="X140" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Y140" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -20143,7 +20143,7 @@
         </is>
       </c>
       <c r="V176" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W176" t="n">
         <v>0</v>
@@ -26822,9 +26822,7 @@
           <t>2026-03-19</t>
         </is>
       </c>
-      <c r="V234" t="n">
-        <v>1</v>
-      </c>
+      <c r="V234" t="inlineStr"/>
       <c r="W234" t="n">
         <v>0</v>
       </c>
@@ -26940,7 +26938,7 @@
         </is>
       </c>
       <c r="V235" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="W235" t="n">
         <v>0</v>
@@ -27057,7 +27055,7 @@
         </is>
       </c>
       <c r="V236" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="W236" t="n">
         <v>0</v>
@@ -29693,9 +29691,7 @@
           <t>2026-04-28</t>
         </is>
       </c>
-      <c r="V259" t="n">
-        <v>1</v>
-      </c>
+      <c r="V259" t="inlineStr"/>
       <c r="W259" t="n">
         <v>0</v>
       </c>
@@ -29927,9 +29923,7 @@
           <t>2026-05-08</t>
         </is>
       </c>
-      <c r="V261" t="n">
-        <v>1</v>
-      </c>
+      <c r="V261" t="inlineStr"/>
       <c r="W261" t="n">
         <v>0</v>
       </c>

</xml_diff>